<commit_message>
add missing DOIs; add Policy Impact metrics
</commit_message>
<xml_diff>
--- a/data/research_metrics_2022-2024.xlsx
+++ b/data/research_metrics_2022-2024.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rosscunning/Projects/research_metrics/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{006E454A-0623-A341-AECF-7AB2722872B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0621D2FF-5B49-C244-82D6-2A7D28D309BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3300" yWindow="2540" windowWidth="34820" windowHeight="16940" xr2:uid="{56BC3C1D-7923-7740-B0BC-17B88C6D3DFD}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AJ$1</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -30,6 +30,7 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -583,9 +584,6 @@
     <t>Lynch A.J., R.I. Arthur, C. Baigun, J.E. Claussen, K.Kangur, A. Koning, K.J. Murchie, B.J.E. Myers, G.L. Stokes, R.W. Tingley, S-J Youn. 2022. Societal Values of Inland Fishes. Pages 475-490 in T. Mehner and K. Tockner (Eds.) C.M. Febria and G. Krantzberg (section Eds.), Encyclopedia of Inland Waters, Second Edition. Elsevier, Amsterdam, Netherlands.</t>
   </si>
   <si>
-    <t>https://www.sciencedirect.com/science/article/pii/B978012819166800030X?via%3Dihub</t>
-  </si>
-  <si>
     <t>Two interns started in June, one full-time and one part-time</t>
   </si>
   <si>
@@ -2135,13 +2133,16 @@
   </si>
   <si>
     <t>Academic</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1016/B978-0-12-819166-8.00030-X</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2152,6 +2153,14 @@
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2174,17 +2183,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2201,9 +2213,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2241,7 +2253,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2347,7 +2359,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2489,7 +2501,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2503,118 +2515,119 @@
     <col min="2" max="2" width="14.1640625" customWidth="1"/>
     <col min="3" max="3" width="16.5" customWidth="1"/>
     <col min="18" max="18" width="40.6640625" customWidth="1"/>
+    <col min="23" max="23" width="94.83203125" customWidth="1"/>
     <col min="30" max="30" width="23.6640625" customWidth="1"/>
     <col min="31" max="31" width="17.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>661</v>
+      </c>
+      <c r="B1" t="s">
         <v>662</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>663</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>664</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>665</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>666</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>667</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>668</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>669</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>670</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>671</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>672</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>673</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>674</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>675</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>676</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>677</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>678</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>679</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>680</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>681</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>682</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>683</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>684</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>685</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>686</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>687</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>688</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" t="s">
         <v>689</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AD1" t="s">
         <v>690</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AE1" t="s">
         <v>691</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AF1" t="s">
         <v>692</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AG1" t="s">
         <v>693</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AH1" t="s">
         <v>694</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AI1" t="s">
         <v>695</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AJ1" t="s">
         <v>696</v>
-      </c>
-      <c r="AJ1" t="s">
-        <v>697</v>
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.2">
@@ -2658,7 +2671,7 @@
         <v>49</v>
       </c>
       <c r="R2" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="AD2">
         <v>300</v>
@@ -2667,7 +2680,7 @@
         <v>150</v>
       </c>
       <c r="AJ2" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
     </row>
     <row r="3" spans="1:36" x14ac:dyDescent="0.2">
@@ -2714,7 +2727,7 @@
         <v>43</v>
       </c>
       <c r="AJ3" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="4" spans="1:36" x14ac:dyDescent="0.2">
@@ -2758,7 +2771,7 @@
         <v>43</v>
       </c>
       <c r="AJ4" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
     </row>
     <row r="5" spans="1:36" x14ac:dyDescent="0.2">
@@ -2849,10 +2862,10 @@
         <v>12</v>
       </c>
       <c r="P6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="R6" s="4" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="AD6">
         <v>8</v>
@@ -2861,7 +2874,7 @@
         <v>40</v>
       </c>
       <c r="AJ6" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.2">
@@ -2902,10 +2915,10 @@
         <v>12</v>
       </c>
       <c r="P7" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="R7" s="4" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="AD7">
         <v>3</v>
@@ -2914,7 +2927,7 @@
         <v>30</v>
       </c>
       <c r="AJ7" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="8" spans="1:36" x14ac:dyDescent="0.2">
@@ -2958,10 +2971,10 @@
         <v>12</v>
       </c>
       <c r="P8" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="R8" s="4" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="AD8">
         <v>60</v>
@@ -2970,7 +2983,7 @@
         <v>30</v>
       </c>
       <c r="AJ8" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
     </row>
     <row r="9" spans="1:36" x14ac:dyDescent="0.2">
@@ -2984,10 +2997,10 @@
         <v>44906.843425925923</v>
       </c>
       <c r="D9" t="s">
+        <v>389</v>
+      </c>
+      <c r="E9" t="s">
         <v>390</v>
-      </c>
-      <c r="E9" t="s">
-        <v>391</v>
       </c>
       <c r="F9" t="s">
         <v>2</v>
@@ -3014,7 +3027,7 @@
         <v>22</v>
       </c>
       <c r="AJ9" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="10" spans="1:36" x14ac:dyDescent="0.2">
@@ -3028,10 +3041,10 @@
         <v>44906.84275462963</v>
       </c>
       <c r="D10" t="s">
+        <v>389</v>
+      </c>
+      <c r="E10" t="s">
         <v>390</v>
-      </c>
-      <c r="E10" t="s">
-        <v>391</v>
       </c>
       <c r="F10" t="s">
         <v>2</v>
@@ -3058,7 +3071,7 @@
         <v>20</v>
       </c>
       <c r="AJ10" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="11" spans="1:36" x14ac:dyDescent="0.2">
@@ -3108,7 +3121,7 @@
         <v>12</v>
       </c>
       <c r="AJ11" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="12" spans="1:36" x14ac:dyDescent="0.2">
@@ -3208,7 +3221,7 @@
         <v>2</v>
       </c>
       <c r="AJ13" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="14" spans="1:36" x14ac:dyDescent="0.2">
@@ -3249,7 +3262,7 @@
         <v>2</v>
       </c>
       <c r="AJ14" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="15" spans="1:36" x14ac:dyDescent="0.2">
@@ -3290,7 +3303,7 @@
         <v>2</v>
       </c>
       <c r="AJ15" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="16" spans="1:36" x14ac:dyDescent="0.2">
@@ -3337,7 +3350,7 @@
         <v>2</v>
       </c>
       <c r="AJ16" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
     </row>
     <row r="17" spans="1:36" x14ac:dyDescent="0.2">
@@ -3760,7 +3773,7 @@
         <v>1</v>
       </c>
       <c r="AJ25" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="26" spans="1:36" x14ac:dyDescent="0.2">
@@ -3816,7 +3829,7 @@
         <v>1</v>
       </c>
       <c r="AJ26" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="27" spans="1:36" x14ac:dyDescent="0.2">
@@ -3866,7 +3879,7 @@
         <v>119</v>
       </c>
       <c r="AD27" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="AE27">
         <v>1</v>
@@ -3919,7 +3932,7 @@
         <v>119</v>
       </c>
       <c r="AD28" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="AE28">
         <v>1</v>
@@ -3975,7 +3988,7 @@
         <v>1</v>
       </c>
       <c r="AJ29" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="30" spans="1:36" x14ac:dyDescent="0.2">
@@ -4022,7 +4035,7 @@
         <v>1</v>
       </c>
       <c r="AJ30" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="31" spans="1:36" x14ac:dyDescent="0.2">
@@ -4036,10 +4049,10 @@
         <v>44906.820671296293</v>
       </c>
       <c r="D31" t="s">
+        <v>389</v>
+      </c>
+      <c r="E31" t="s">
         <v>390</v>
-      </c>
-      <c r="E31" t="s">
-        <v>391</v>
       </c>
       <c r="F31" t="s">
         <v>2</v>
@@ -4072,7 +4085,7 @@
         <v>1</v>
       </c>
       <c r="AJ31" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="32" spans="1:36" x14ac:dyDescent="0.2">
@@ -4086,10 +4099,10 @@
         <v>44906.828553240739</v>
       </c>
       <c r="D32" t="s">
+        <v>389</v>
+      </c>
+      <c r="E32" t="s">
         <v>390</v>
-      </c>
-      <c r="E32" t="s">
-        <v>391</v>
       </c>
       <c r="F32" t="s">
         <v>2</v>
@@ -4122,7 +4135,7 @@
         <v>1</v>
       </c>
       <c r="AJ32" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="33" spans="1:36" x14ac:dyDescent="0.2">
@@ -4172,7 +4185,7 @@
         <v>1</v>
       </c>
       <c r="AJ33" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
     </row>
     <row r="34" spans="1:36" x14ac:dyDescent="0.2">
@@ -4219,7 +4232,7 @@
         <v>1</v>
       </c>
       <c r="AJ34" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="35" spans="1:36" x14ac:dyDescent="0.2">
@@ -4266,7 +4279,7 @@
         <v>1</v>
       </c>
       <c r="AJ35" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
     </row>
     <row r="36" spans="1:36" x14ac:dyDescent="0.2">
@@ -4322,7 +4335,7 @@
         <v>1</v>
       </c>
       <c r="AJ36" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
     </row>
     <row r="37" spans="1:36" x14ac:dyDescent="0.2">
@@ -4366,7 +4379,7 @@
         <v>12</v>
       </c>
       <c r="P37" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="R37" t="s">
         <v>119</v>
@@ -4378,7 +4391,7 @@
         <v>0</v>
       </c>
       <c r="AJ37" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="38" spans="1:36" x14ac:dyDescent="0.2">
@@ -5445,7 +5458,7 @@
         <v>18</v>
       </c>
       <c r="AJ59" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="60" spans="1:36" x14ac:dyDescent="0.2">
@@ -5489,13 +5502,13 @@
         <v>12</v>
       </c>
       <c r="P60" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="R60" t="s">
         <v>18</v>
       </c>
       <c r="AJ60" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="61" spans="1:36" x14ac:dyDescent="0.2">
@@ -5542,7 +5555,7 @@
         <v>18</v>
       </c>
       <c r="AJ61" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="62" spans="1:36" x14ac:dyDescent="0.2">
@@ -5586,13 +5599,13 @@
         <v>12</v>
       </c>
       <c r="P62" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="R62" t="s">
         <v>18</v>
       </c>
       <c r="AJ62" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="63" spans="1:36" x14ac:dyDescent="0.2">
@@ -5636,13 +5649,13 @@
         <v>12</v>
       </c>
       <c r="P63" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="R63" t="s">
         <v>18</v>
       </c>
       <c r="AJ63" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="64" spans="1:36" x14ac:dyDescent="0.2">
@@ -5692,7 +5705,7 @@
         <v>18</v>
       </c>
       <c r="AJ64" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="65" spans="1:36" x14ac:dyDescent="0.2">
@@ -5736,7 +5749,7 @@
         <v>18</v>
       </c>
       <c r="AJ65" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="66" spans="1:36" x14ac:dyDescent="0.2">
@@ -5780,13 +5793,13 @@
         <v>12</v>
       </c>
       <c r="P66" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="R66" t="s">
         <v>18</v>
       </c>
       <c r="AJ66" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="67" spans="1:36" x14ac:dyDescent="0.2">
@@ -5836,7 +5849,7 @@
         <v>18</v>
       </c>
       <c r="AJ67" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="68" spans="1:36" x14ac:dyDescent="0.2">
@@ -5880,13 +5893,13 @@
         <v>12</v>
       </c>
       <c r="P68" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="R68" t="s">
         <v>18</v>
       </c>
       <c r="AJ68" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="69" spans="1:36" x14ac:dyDescent="0.2">
@@ -5933,7 +5946,7 @@
         <v>18</v>
       </c>
       <c r="AJ69" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="70" spans="1:36" x14ac:dyDescent="0.2">
@@ -5974,13 +5987,13 @@
         <v>12</v>
       </c>
       <c r="P70" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="R70" t="s">
         <v>18</v>
       </c>
       <c r="AJ70" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="71" spans="1:36" x14ac:dyDescent="0.2">
@@ -6030,7 +6043,7 @@
         <v>18</v>
       </c>
       <c r="AJ71" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="72" spans="1:36" x14ac:dyDescent="0.2">
@@ -6080,7 +6093,7 @@
         <v>18</v>
       </c>
       <c r="AJ72" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="73" spans="1:36" x14ac:dyDescent="0.2">
@@ -6130,7 +6143,7 @@
         <v>18</v>
       </c>
       <c r="AJ73" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="74" spans="1:36" x14ac:dyDescent="0.2">
@@ -6180,7 +6193,7 @@
         <v>18</v>
       </c>
       <c r="AJ74" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="75" spans="1:36" x14ac:dyDescent="0.2">
@@ -6230,7 +6243,7 @@
         <v>18</v>
       </c>
       <c r="AJ75" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="76" spans="1:36" x14ac:dyDescent="0.2">
@@ -6280,7 +6293,7 @@
         <v>18</v>
       </c>
       <c r="AJ76" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="77" spans="1:36" x14ac:dyDescent="0.2">
@@ -6327,7 +6340,7 @@
         <v>18</v>
       </c>
       <c r="AJ77" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="78" spans="1:36" x14ac:dyDescent="0.2">
@@ -6377,7 +6390,7 @@
         <v>18</v>
       </c>
       <c r="AJ78" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="79" spans="1:36" x14ac:dyDescent="0.2">
@@ -6427,7 +6440,7 @@
         <v>18</v>
       </c>
       <c r="AJ79" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="80" spans="1:36" x14ac:dyDescent="0.2">
@@ -6471,7 +6484,7 @@
         <v>18</v>
       </c>
       <c r="AJ80" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="81" spans="1:36" x14ac:dyDescent="0.2">
@@ -6515,13 +6528,13 @@
         <v>12</v>
       </c>
       <c r="P81" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="R81" t="s">
         <v>18</v>
       </c>
       <c r="AJ81" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="82" spans="1:36" x14ac:dyDescent="0.2">
@@ -6571,7 +6584,7 @@
         <v>18</v>
       </c>
       <c r="AJ82" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="83" spans="1:36" x14ac:dyDescent="0.2">
@@ -6621,7 +6634,7 @@
         <v>18</v>
       </c>
       <c r="AJ83" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="84" spans="1:36" x14ac:dyDescent="0.2">
@@ -6635,10 +6648,10 @@
         <v>44906.81177083333</v>
       </c>
       <c r="D84" t="s">
+        <v>389</v>
+      </c>
+      <c r="E84" t="s">
         <v>390</v>
-      </c>
-      <c r="E84" t="s">
-        <v>391</v>
       </c>
       <c r="F84" t="s">
         <v>2</v>
@@ -6668,7 +6681,7 @@
         <v>18</v>
       </c>
       <c r="AJ84" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="85" spans="1:36" x14ac:dyDescent="0.2">
@@ -6682,10 +6695,10 @@
         <v>44906.834178240744</v>
       </c>
       <c r="D85" t="s">
+        <v>389</v>
+      </c>
+      <c r="E85" t="s">
         <v>390</v>
-      </c>
-      <c r="E85" t="s">
-        <v>391</v>
       </c>
       <c r="F85" t="s">
         <v>2</v>
@@ -6709,13 +6722,13 @@
         <v>12</v>
       </c>
       <c r="P85" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="R85" t="s">
         <v>18</v>
       </c>
       <c r="AJ85" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="86" spans="1:36" x14ac:dyDescent="0.2">
@@ -6765,7 +6778,7 @@
         <v>18</v>
       </c>
       <c r="AJ86" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="87" spans="1:36" x14ac:dyDescent="0.2">
@@ -6809,7 +6822,7 @@
         <v>18</v>
       </c>
       <c r="AJ87" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="88" spans="1:36" x14ac:dyDescent="0.2">
@@ -6850,13 +6863,13 @@
         <v>12</v>
       </c>
       <c r="P88" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="R88" t="s">
         <v>18</v>
       </c>
       <c r="AJ88" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="89" spans="1:36" x14ac:dyDescent="0.2">
@@ -6897,13 +6910,13 @@
         <v>12</v>
       </c>
       <c r="P89" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="R89" t="s">
         <v>18</v>
       </c>
       <c r="AJ89" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="90" spans="1:36" x14ac:dyDescent="0.2">
@@ -6944,13 +6957,13 @@
         <v>12</v>
       </c>
       <c r="P90" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="R90" t="s">
         <v>18</v>
       </c>
       <c r="AJ90" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="91" spans="1:36" x14ac:dyDescent="0.2">
@@ -6991,13 +7004,13 @@
         <v>12</v>
       </c>
       <c r="P91" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="R91" t="s">
         <v>18</v>
       </c>
       <c r="AJ91" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="92" spans="1:36" x14ac:dyDescent="0.2">
@@ -7038,13 +7051,13 @@
         <v>12</v>
       </c>
       <c r="P92" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="R92" t="s">
         <v>18</v>
       </c>
       <c r="AJ92" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="93" spans="1:36" x14ac:dyDescent="0.2">
@@ -7088,7 +7101,7 @@
         <v>18</v>
       </c>
       <c r="AJ93" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="94" spans="1:36" x14ac:dyDescent="0.2">
@@ -7129,7 +7142,7 @@
         <v>18</v>
       </c>
       <c r="AJ94" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="95" spans="1:36" x14ac:dyDescent="0.2">
@@ -7179,7 +7192,7 @@
         <v>18</v>
       </c>
       <c r="AJ95" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="96" spans="1:36" x14ac:dyDescent="0.2">
@@ -7229,7 +7242,7 @@
         <v>18</v>
       </c>
       <c r="AJ96" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="97" spans="1:36" x14ac:dyDescent="0.2">
@@ -7279,7 +7292,7 @@
         <v>18</v>
       </c>
       <c r="AJ97" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="98" spans="1:36" x14ac:dyDescent="0.2">
@@ -7323,13 +7336,13 @@
         <v>12</v>
       </c>
       <c r="P98" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="R98" t="s">
         <v>18</v>
       </c>
       <c r="AJ98" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="99" spans="1:36" x14ac:dyDescent="0.2">
@@ -7373,13 +7386,13 @@
         <v>12</v>
       </c>
       <c r="P99" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="R99" t="s">
         <v>18</v>
       </c>
       <c r="AJ99" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="100" spans="1:36" x14ac:dyDescent="0.2">
@@ -7429,7 +7442,7 @@
         <v>18</v>
       </c>
       <c r="AJ100" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="101" spans="1:36" x14ac:dyDescent="0.2">
@@ -7473,13 +7486,13 @@
         <v>12</v>
       </c>
       <c r="P101" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="R101" t="s">
         <v>18</v>
       </c>
       <c r="AJ101" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="102" spans="1:36" x14ac:dyDescent="0.2">
@@ -7529,7 +7542,7 @@
         <v>18</v>
       </c>
       <c r="AJ102" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="103" spans="1:36" x14ac:dyDescent="0.2">
@@ -7579,7 +7592,7 @@
         <v>18</v>
       </c>
       <c r="AJ103" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="104" spans="1:36" x14ac:dyDescent="0.2">
@@ -7629,7 +7642,7 @@
         <v>18</v>
       </c>
       <c r="AJ104" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
     </row>
     <row r="105" spans="1:36" x14ac:dyDescent="0.2">
@@ -7676,7 +7689,7 @@
         <v>18</v>
       </c>
       <c r="AJ105" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
     </row>
     <row r="106" spans="1:36" x14ac:dyDescent="0.2">
@@ -7726,7 +7739,7 @@
         <v>18</v>
       </c>
       <c r="AJ106" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="107" spans="1:36" x14ac:dyDescent="0.2">
@@ -7776,7 +7789,7 @@
         <v>18</v>
       </c>
       <c r="AJ107" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
     </row>
     <row r="108" spans="1:36" x14ac:dyDescent="0.2">
@@ -7917,7 +7930,7 @@
         <v>18</v>
       </c>
       <c r="AJ110" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="111" spans="1:36" x14ac:dyDescent="0.2">
@@ -7961,13 +7974,13 @@
         <v>12</v>
       </c>
       <c r="P111" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="R111" t="s">
         <v>18</v>
       </c>
       <c r="AJ111" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
     </row>
     <row r="112" spans="1:36" x14ac:dyDescent="0.2">
@@ -8014,7 +8027,7 @@
         <v>18</v>
       </c>
       <c r="AJ112" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="113" spans="1:36" x14ac:dyDescent="0.2">
@@ -8058,13 +8071,13 @@
         <v>12</v>
       </c>
       <c r="P113" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="R113" t="s">
         <v>18</v>
       </c>
       <c r="AJ113" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
     </row>
     <row r="114" spans="1:36" x14ac:dyDescent="0.2">
@@ -8111,7 +8124,7 @@
         <v>18</v>
       </c>
       <c r="AJ114" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="115" spans="1:36" x14ac:dyDescent="0.2">
@@ -8155,7 +8168,7 @@
         <v>18</v>
       </c>
       <c r="AJ115" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
     </row>
     <row r="116" spans="1:36" x14ac:dyDescent="0.2">
@@ -8202,7 +8215,7 @@
         <v>18</v>
       </c>
       <c r="AJ116" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
     </row>
     <row r="117" spans="1:36" x14ac:dyDescent="0.2">
@@ -8243,13 +8256,13 @@
         <v>12</v>
       </c>
       <c r="P117" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="R117" t="s">
         <v>18</v>
       </c>
       <c r="AJ117" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
     </row>
     <row r="118" spans="1:36" x14ac:dyDescent="0.2">
@@ -8293,13 +8306,13 @@
         <v>12</v>
       </c>
       <c r="P118" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="R118" t="s">
         <v>18</v>
       </c>
       <c r="AJ118" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="119" spans="1:36" x14ac:dyDescent="0.2">
@@ -8343,13 +8356,13 @@
         <v>12</v>
       </c>
       <c r="P119" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="R119" t="s">
         <v>18</v>
       </c>
       <c r="AJ119" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
     </row>
     <row r="120" spans="1:36" x14ac:dyDescent="0.2">
@@ -8399,7 +8412,7 @@
         <v>18</v>
       </c>
       <c r="AJ120" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
     </row>
     <row r="121" spans="1:36" x14ac:dyDescent="0.2">
@@ -8443,13 +8456,13 @@
         <v>12</v>
       </c>
       <c r="P121" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="R121" t="s">
         <v>18</v>
       </c>
       <c r="AJ121" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
     </row>
     <row r="122" spans="1:36" x14ac:dyDescent="0.2">
@@ -8499,7 +8512,7 @@
         <v>18</v>
       </c>
       <c r="AJ122" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
     </row>
     <row r="123" spans="1:36" x14ac:dyDescent="0.2">
@@ -8537,13 +8550,13 @@
         <v>12</v>
       </c>
       <c r="P123" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="R123" t="s">
         <v>18</v>
       </c>
       <c r="AJ123" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
     </row>
     <row r="124" spans="1:36" x14ac:dyDescent="0.2">
@@ -8593,7 +8606,7 @@
         <v>18</v>
       </c>
       <c r="AJ124" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
     </row>
     <row r="125" spans="1:36" x14ac:dyDescent="0.2">
@@ -8637,13 +8650,13 @@
         <v>12</v>
       </c>
       <c r="P125" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="R125" t="s">
         <v>18</v>
       </c>
       <c r="AJ125" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
     </row>
     <row r="126" spans="1:36" x14ac:dyDescent="0.2">
@@ -8690,7 +8703,7 @@
         <v>1600</v>
       </c>
       <c r="AJ126" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="127" spans="1:36" x14ac:dyDescent="0.2">
@@ -8734,7 +8747,7 @@
         <v>366</v>
       </c>
       <c r="AJ127" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="128" spans="1:36" x14ac:dyDescent="0.2">
@@ -8951,7 +8964,7 @@
         <v>78</v>
       </c>
       <c r="AJ132" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="133" spans="1:36" x14ac:dyDescent="0.2">
@@ -8995,7 +9008,7 @@
         <v>78</v>
       </c>
       <c r="AJ133" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="134" spans="1:36" x14ac:dyDescent="0.2">
@@ -9042,7 +9055,7 @@
         <v>78</v>
       </c>
       <c r="AJ134" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="135" spans="1:36" x14ac:dyDescent="0.2">
@@ -9080,13 +9093,13 @@
         <v>12</v>
       </c>
       <c r="P135" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R135" t="s">
         <v>78</v>
       </c>
       <c r="AJ135" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="136" spans="1:36" x14ac:dyDescent="0.2">
@@ -9127,13 +9140,13 @@
         <v>12</v>
       </c>
       <c r="P136" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="R136" t="s">
         <v>78</v>
       </c>
       <c r="AJ136" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="137" spans="1:36" x14ac:dyDescent="0.2">
@@ -9174,7 +9187,7 @@
         <v>78</v>
       </c>
       <c r="AJ137" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="138" spans="1:36" x14ac:dyDescent="0.2">
@@ -9218,7 +9231,7 @@
         <v>78</v>
       </c>
       <c r="AJ138" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="139" spans="1:36" x14ac:dyDescent="0.2">
@@ -9262,7 +9275,7 @@
         <v>78</v>
       </c>
       <c r="AJ139" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="140" spans="1:36" x14ac:dyDescent="0.2">
@@ -9303,13 +9316,13 @@
         <v>12</v>
       </c>
       <c r="P140" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="R140" t="s">
         <v>78</v>
       </c>
       <c r="AJ140" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
     </row>
     <row r="141" spans="1:36" x14ac:dyDescent="0.2">
@@ -9350,13 +9363,13 @@
         <v>12</v>
       </c>
       <c r="P141" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="R141" t="s">
         <v>78</v>
       </c>
       <c r="AJ141" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
     </row>
     <row r="142" spans="1:36" x14ac:dyDescent="0.2">
@@ -9400,7 +9413,7 @@
         <v>78</v>
       </c>
       <c r="AJ142" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
     </row>
     <row r="143" spans="1:36" x14ac:dyDescent="0.2">
@@ -9441,7 +9454,7 @@
         <v>78</v>
       </c>
       <c r="AJ143" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="144" spans="1:36" x14ac:dyDescent="0.2">
@@ -9482,7 +9495,7 @@
         <v>78</v>
       </c>
       <c r="AJ144" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="145" spans="1:36" x14ac:dyDescent="0.2">
@@ -9564,7 +9577,7 @@
         <v>78</v>
       </c>
       <c r="AJ146" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
     </row>
     <row r="147" spans="1:36" x14ac:dyDescent="0.2">
@@ -9605,13 +9618,13 @@
         <v>12</v>
       </c>
       <c r="P147" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="R147" t="s">
         <v>78</v>
       </c>
       <c r="AJ147" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="148" spans="1:36" x14ac:dyDescent="0.2">
@@ -10210,7 +10223,7 @@
         <v>74</v>
       </c>
       <c r="AJ160" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="161" spans="1:36" x14ac:dyDescent="0.2">
@@ -10254,7 +10267,7 @@
         <v>150</v>
       </c>
       <c r="AJ161" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="162" spans="1:36" x14ac:dyDescent="0.2">
@@ -10298,7 +10311,7 @@
         <v>150</v>
       </c>
       <c r="AJ162" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="163" spans="1:36" x14ac:dyDescent="0.2">
@@ -10339,16 +10352,16 @@
         <v>12</v>
       </c>
       <c r="P163" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="R163" t="s">
         <v>55</v>
       </c>
       <c r="AC163" t="s">
+        <v>202</v>
+      </c>
+      <c r="AJ163" t="s">
         <v>203</v>
-      </c>
-      <c r="AJ163" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="164" spans="1:36" x14ac:dyDescent="0.2">
@@ -10392,10 +10405,10 @@
         <v>55</v>
       </c>
       <c r="AC164" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AJ164" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="165" spans="1:36" x14ac:dyDescent="0.2">
@@ -10436,10 +10449,10 @@
         <v>55</v>
       </c>
       <c r="AC165" t="s">
+        <v>205</v>
+      </c>
+      <c r="AJ165" t="s">
         <v>206</v>
-      </c>
-      <c r="AJ165" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="166" spans="1:36" x14ac:dyDescent="0.2">
@@ -10483,10 +10496,10 @@
         <v>55</v>
       </c>
       <c r="AC166" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AJ166" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="167" spans="1:36" x14ac:dyDescent="0.2">
@@ -10527,10 +10540,10 @@
         <v>55</v>
       </c>
       <c r="AC167" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AJ167" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="168" spans="1:36" x14ac:dyDescent="0.2">
@@ -10574,7 +10587,7 @@
         <v>157</v>
       </c>
       <c r="AJ168" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="169" spans="1:36" x14ac:dyDescent="0.2">
@@ -10615,13 +10628,13 @@
         <v>5</v>
       </c>
       <c r="Q169" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="R169" t="s">
         <v>55</v>
       </c>
       <c r="AC169" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="170" spans="1:36" x14ac:dyDescent="0.2">
@@ -10665,7 +10678,7 @@
         <v>157</v>
       </c>
       <c r="AJ170" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="171" spans="1:36" x14ac:dyDescent="0.2">
@@ -10712,7 +10725,7 @@
         <v>56</v>
       </c>
       <c r="AJ171" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="172" spans="1:36" x14ac:dyDescent="0.2">
@@ -10759,7 +10772,7 @@
         <v>56</v>
       </c>
       <c r="AJ172" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="173" spans="1:36" x14ac:dyDescent="0.2">
@@ -10806,7 +10819,7 @@
         <v>56</v>
       </c>
       <c r="AJ173" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="174" spans="1:36" x14ac:dyDescent="0.2">
@@ -10856,10 +10869,10 @@
         <v>55</v>
       </c>
       <c r="AC174" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="AJ174" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="175" spans="1:36" x14ac:dyDescent="0.2">
@@ -10912,7 +10925,7 @@
         <v>150</v>
       </c>
       <c r="AJ175" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="176" spans="1:36" x14ac:dyDescent="0.2">
@@ -10965,7 +10978,7 @@
         <v>150</v>
       </c>
       <c r="AJ176" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="177" spans="1:36" x14ac:dyDescent="0.2">
@@ -11091,7 +11104,7 @@
         <v>74</v>
       </c>
       <c r="AJ179" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="180" spans="1:36" x14ac:dyDescent="0.2">
@@ -11138,10 +11151,10 @@
         <v>55</v>
       </c>
       <c r="AC180" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="AJ180" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="181" spans="1:36" x14ac:dyDescent="0.2">
@@ -11155,10 +11168,10 @@
         <v>44906.796307870369</v>
       </c>
       <c r="D181" t="s">
+        <v>389</v>
+      </c>
+      <c r="E181" t="s">
         <v>390</v>
-      </c>
-      <c r="E181" t="s">
-        <v>391</v>
       </c>
       <c r="F181" t="s">
         <v>2</v>
@@ -11191,7 +11204,7 @@
         <v>74</v>
       </c>
       <c r="AJ181" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="182" spans="1:36" x14ac:dyDescent="0.2">
@@ -11205,10 +11218,10 @@
         <v>44906.80269675926</v>
       </c>
       <c r="D182" t="s">
+        <v>389</v>
+      </c>
+      <c r="E182" t="s">
         <v>390</v>
-      </c>
-      <c r="E182" t="s">
-        <v>391</v>
       </c>
       <c r="F182" t="s">
         <v>2</v>
@@ -11232,7 +11245,7 @@
         <v>55</v>
       </c>
       <c r="AJ182" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="183" spans="1:36" x14ac:dyDescent="0.2">
@@ -11246,10 +11259,10 @@
         <v>44906.803738425922</v>
       </c>
       <c r="D183" t="s">
+        <v>389</v>
+      </c>
+      <c r="E183" t="s">
         <v>390</v>
-      </c>
-      <c r="E183" t="s">
-        <v>391</v>
       </c>
       <c r="F183" t="s">
         <v>2</v>
@@ -11279,7 +11292,7 @@
         <v>74</v>
       </c>
       <c r="AJ183" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="184" spans="1:36" x14ac:dyDescent="0.2">
@@ -11293,10 +11306,10 @@
         <v>44906.805231481485</v>
       </c>
       <c r="D184" t="s">
+        <v>389</v>
+      </c>
+      <c r="E184" t="s">
         <v>390</v>
-      </c>
-      <c r="E184" t="s">
-        <v>391</v>
       </c>
       <c r="F184" t="s">
         <v>2</v>
@@ -11326,7 +11339,7 @@
         <v>150</v>
       </c>
       <c r="AJ184" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="185" spans="1:36" x14ac:dyDescent="0.2">
@@ -11340,10 +11353,10 @@
         <v>44906.81013888889</v>
       </c>
       <c r="D185" t="s">
+        <v>389</v>
+      </c>
+      <c r="E185" t="s">
         <v>390</v>
-      </c>
-      <c r="E185" t="s">
-        <v>391</v>
       </c>
       <c r="F185" t="s">
         <v>2</v>
@@ -11367,7 +11380,7 @@
         <v>55</v>
       </c>
       <c r="AJ185" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="186" spans="1:36" x14ac:dyDescent="0.2">
@@ -11381,10 +11394,10 @@
         <v>44906.813506944447</v>
       </c>
       <c r="D186" t="s">
+        <v>389</v>
+      </c>
+      <c r="E186" t="s">
         <v>390</v>
-      </c>
-      <c r="E186" t="s">
-        <v>391</v>
       </c>
       <c r="F186" t="s">
         <v>2</v>
@@ -11411,7 +11424,7 @@
         <v>56</v>
       </c>
       <c r="AJ186" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="187" spans="1:36" x14ac:dyDescent="0.2">
@@ -11425,10 +11438,10 @@
         <v>44906.815520833334</v>
       </c>
       <c r="D187" t="s">
+        <v>389</v>
+      </c>
+      <c r="E187" t="s">
         <v>390</v>
-      </c>
-      <c r="E187" t="s">
-        <v>391</v>
       </c>
       <c r="F187" t="s">
         <v>2</v>
@@ -11458,10 +11471,10 @@
         <v>55</v>
       </c>
       <c r="AC187" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="AJ187" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="188" spans="1:36" x14ac:dyDescent="0.2">
@@ -11475,10 +11488,10 @@
         <v>44906.826828703706</v>
       </c>
       <c r="D188" t="s">
+        <v>389</v>
+      </c>
+      <c r="E188" t="s">
         <v>390</v>
-      </c>
-      <c r="E188" t="s">
-        <v>391</v>
       </c>
       <c r="F188" t="s">
         <v>2</v>
@@ -11508,7 +11521,7 @@
         <v>55</v>
       </c>
       <c r="AJ188" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="189" spans="1:36" x14ac:dyDescent="0.2">
@@ -11549,10 +11562,10 @@
         <v>55</v>
       </c>
       <c r="AC189" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AJ189" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="190" spans="1:36" x14ac:dyDescent="0.2">
@@ -11681,7 +11694,7 @@
         <v>157</v>
       </c>
       <c r="AJ192" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="193" spans="1:36" x14ac:dyDescent="0.2">
@@ -11725,7 +11738,7 @@
         <v>74</v>
       </c>
       <c r="AJ193" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="194" spans="1:36" x14ac:dyDescent="0.2">
@@ -11766,7 +11779,7 @@
         <v>12</v>
       </c>
       <c r="P194" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="R194" t="s">
         <v>55</v>
@@ -11775,7 +11788,7 @@
         <v>150</v>
       </c>
       <c r="AJ194" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="195" spans="1:36" x14ac:dyDescent="0.2">
@@ -11819,7 +11832,7 @@
         <v>74</v>
       </c>
       <c r="AJ195" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="196" spans="1:36" x14ac:dyDescent="0.2">
@@ -11863,10 +11876,10 @@
         <v>55</v>
       </c>
       <c r="AC196" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AJ196" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
     <row r="197" spans="1:36" x14ac:dyDescent="0.2">
@@ -11913,7 +11926,7 @@
         <v>157</v>
       </c>
       <c r="AJ197" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
     </row>
     <row r="198" spans="1:36" x14ac:dyDescent="0.2">
@@ -11960,7 +11973,7 @@
         <v>157</v>
       </c>
       <c r="AJ198" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="199" spans="1:36" x14ac:dyDescent="0.2">
@@ -12010,7 +12023,7 @@
         <v>157</v>
       </c>
       <c r="AJ199" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
     </row>
     <row r="200" spans="1:36" x14ac:dyDescent="0.2">
@@ -12057,7 +12070,7 @@
         <v>157</v>
       </c>
       <c r="AJ200" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
     </row>
     <row r="201" spans="1:36" x14ac:dyDescent="0.2">
@@ -12104,7 +12117,7 @@
         <v>150</v>
       </c>
       <c r="AJ201" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
     </row>
     <row r="202" spans="1:36" x14ac:dyDescent="0.2">
@@ -12359,7 +12372,7 @@
         <v>157</v>
       </c>
       <c r="AJ207" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
     </row>
     <row r="208" spans="1:36" x14ac:dyDescent="0.2">
@@ -12406,7 +12419,7 @@
         <v>150</v>
       </c>
       <c r="AJ208" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
     </row>
     <row r="209" spans="1:36" x14ac:dyDescent="0.2">
@@ -12456,7 +12469,7 @@
         <v>150</v>
       </c>
       <c r="AJ209" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="210" spans="1:36" x14ac:dyDescent="0.2">
@@ -12497,10 +12510,10 @@
         <v>55</v>
       </c>
       <c r="AC210" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AJ210" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="211" spans="1:36" x14ac:dyDescent="0.2">
@@ -12541,7 +12554,7 @@
         <v>55</v>
       </c>
       <c r="AC211" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="212" spans="1:36" x14ac:dyDescent="0.2">
@@ -12582,7 +12595,7 @@
         <v>55</v>
       </c>
       <c r="AC212" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="213" spans="1:36" x14ac:dyDescent="0.2">
@@ -12623,10 +12636,10 @@
         <v>55</v>
       </c>
       <c r="AC213" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AJ213" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
     <row r="214" spans="1:36" x14ac:dyDescent="0.2">
@@ -12667,10 +12680,10 @@
         <v>55</v>
       </c>
       <c r="AC214" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AJ214" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="215" spans="1:36" x14ac:dyDescent="0.2">
@@ -12711,10 +12724,10 @@
         <v>55</v>
       </c>
       <c r="AC215" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AJ215" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
     </row>
     <row r="216" spans="1:36" x14ac:dyDescent="0.2">
@@ -12755,7 +12768,7 @@
         <v>55</v>
       </c>
       <c r="AC216" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="217" spans="1:36" x14ac:dyDescent="0.2">
@@ -12796,10 +12809,10 @@
         <v>55</v>
       </c>
       <c r="AC217" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AJ217" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
     </row>
     <row r="218" spans="1:36" x14ac:dyDescent="0.2">
@@ -12843,7 +12856,7 @@
         <v>74</v>
       </c>
       <c r="AJ218" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
     </row>
     <row r="219" spans="1:36" x14ac:dyDescent="0.2">
@@ -12887,10 +12900,10 @@
         <v>55</v>
       </c>
       <c r="AC219" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AJ219" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
     </row>
     <row r="220" spans="1:36" x14ac:dyDescent="0.2">
@@ -13681,10 +13694,10 @@
         <v>7</v>
       </c>
       <c r="Z235" t="s">
+        <v>192</v>
+      </c>
+      <c r="AA235" t="s">
         <v>193</v>
-      </c>
-      <c r="AA235" t="s">
-        <v>194</v>
       </c>
       <c r="AB235" s="2">
         <v>44686</v>
@@ -13725,10 +13738,10 @@
         <v>7</v>
       </c>
       <c r="Z236" t="s">
+        <v>195</v>
+      </c>
+      <c r="AA236" t="s">
         <v>196</v>
-      </c>
-      <c r="AA236" t="s">
-        <v>197</v>
       </c>
       <c r="AB236" s="2">
         <v>44741</v>
@@ -13775,16 +13788,16 @@
         <v>12</v>
       </c>
       <c r="P237" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="R237" t="s">
         <v>7</v>
       </c>
       <c r="Z237" t="s">
+        <v>210</v>
+      </c>
+      <c r="AA237" t="s">
         <v>211</v>
-      </c>
-      <c r="AA237" t="s">
-        <v>212</v>
       </c>
       <c r="AB237" s="2">
         <v>44733</v>
@@ -13822,10 +13835,10 @@
         <v>7</v>
       </c>
       <c r="Z238" t="s">
+        <v>230</v>
+      </c>
+      <c r="AA238" t="s">
         <v>231</v>
-      </c>
-      <c r="AA238" t="s">
-        <v>232</v>
       </c>
       <c r="AB238" s="2">
         <v>44757</v>
@@ -13875,10 +13888,10 @@
         <v>7</v>
       </c>
       <c r="Z239" t="s">
+        <v>235</v>
+      </c>
+      <c r="AA239" t="s">
         <v>236</v>
-      </c>
-      <c r="AA239" t="s">
-        <v>237</v>
       </c>
       <c r="AB239" s="2">
         <v>44767</v>
@@ -13931,10 +13944,10 @@
         <v>7</v>
       </c>
       <c r="Z240" t="s">
+        <v>256</v>
+      </c>
+      <c r="AJ240" t="s">
         <v>257</v>
-      </c>
-      <c r="AJ240" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="241" spans="1:36" x14ac:dyDescent="0.2">
@@ -13978,16 +13991,16 @@
         <v>12</v>
       </c>
       <c r="P241" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="R241" t="s">
         <v>7</v>
       </c>
       <c r="Z241" t="s">
+        <v>263</v>
+      </c>
+      <c r="AJ241" t="s">
         <v>264</v>
-      </c>
-      <c r="AJ241" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="242" spans="1:36" x14ac:dyDescent="0.2">
@@ -14031,16 +14044,16 @@
         <v>12</v>
       </c>
       <c r="P242" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="R242" t="s">
         <v>7</v>
       </c>
       <c r="Z242" t="s">
+        <v>265</v>
+      </c>
+      <c r="AJ242" t="s">
         <v>266</v>
-      </c>
-      <c r="AJ242" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="243" spans="1:36" x14ac:dyDescent="0.2">
@@ -14084,16 +14097,16 @@
         <v>12</v>
       </c>
       <c r="P243" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="R243" t="s">
         <v>7</v>
       </c>
       <c r="Z243" t="s">
+        <v>271</v>
+      </c>
+      <c r="AJ243" t="s">
         <v>272</v>
-      </c>
-      <c r="AJ243" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="244" spans="1:36" x14ac:dyDescent="0.2">
@@ -14134,16 +14147,16 @@
         <v>12</v>
       </c>
       <c r="P244" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="R244" t="s">
         <v>7</v>
       </c>
       <c r="Z244" t="s">
+        <v>276</v>
+      </c>
+      <c r="AA244" t="s">
         <v>277</v>
-      </c>
-      <c r="AA244" t="s">
-        <v>278</v>
       </c>
       <c r="AB244" s="2">
         <v>44829</v>
@@ -14181,13 +14194,13 @@
         <v>12</v>
       </c>
       <c r="P245" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="R245" t="s">
         <v>7</v>
       </c>
       <c r="Z245" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="AB245" s="2">
         <v>44791</v>
@@ -14231,10 +14244,10 @@
         <v>7</v>
       </c>
       <c r="Z246" t="s">
+        <v>294</v>
+      </c>
+      <c r="AA246" t="s">
         <v>295</v>
-      </c>
-      <c r="AA246" t="s">
-        <v>296</v>
       </c>
       <c r="AB246" s="2">
         <v>44854</v>
@@ -14278,10 +14291,10 @@
         <v>7</v>
       </c>
       <c r="Z247" t="s">
+        <v>296</v>
+      </c>
+      <c r="AA247" t="s">
         <v>297</v>
-      </c>
-      <c r="AA247" t="s">
-        <v>298</v>
       </c>
       <c r="AB247" s="2">
         <v>44855</v>
@@ -14328,16 +14341,16 @@
         <v>12</v>
       </c>
       <c r="P248" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="R248" t="s">
         <v>7</v>
       </c>
       <c r="Z248" t="s">
+        <v>316</v>
+      </c>
+      <c r="AA248" t="s">
         <v>317</v>
-      </c>
-      <c r="AA248" t="s">
-        <v>318</v>
       </c>
       <c r="AB248" s="2">
         <v>44865</v>
@@ -14378,16 +14391,16 @@
         <v>7</v>
       </c>
       <c r="Z249" t="s">
+        <v>329</v>
+      </c>
+      <c r="AA249" t="s">
         <v>330</v>
-      </c>
-      <c r="AA249" t="s">
-        <v>331</v>
       </c>
       <c r="AB249" s="2">
         <v>44873</v>
       </c>
       <c r="AJ249" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="250" spans="1:36" x14ac:dyDescent="0.2">
@@ -14431,16 +14444,16 @@
         <v>12</v>
       </c>
       <c r="P250" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="R250" t="s">
         <v>7</v>
       </c>
       <c r="Z250" t="s">
+        <v>341</v>
+      </c>
+      <c r="AJ250" t="s">
         <v>342</v>
-      </c>
-      <c r="AJ250" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="251" spans="1:36" x14ac:dyDescent="0.2">
@@ -14484,22 +14497,22 @@
         <v>12</v>
       </c>
       <c r="P251" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="R251" t="s">
         <v>7</v>
       </c>
       <c r="Z251" t="s">
+        <v>370</v>
+      </c>
+      <c r="AA251" t="s">
         <v>371</v>
-      </c>
-      <c r="AA251" t="s">
-        <v>372</v>
       </c>
       <c r="AB251" s="2">
         <v>44790</v>
       </c>
       <c r="AJ251" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="252" spans="1:36" x14ac:dyDescent="0.2">
@@ -14534,10 +14547,10 @@
         <v>7</v>
       </c>
       <c r="Z252" t="s">
+        <v>440</v>
+      </c>
+      <c r="AA252" t="s">
         <v>441</v>
-      </c>
-      <c r="AA252" t="s">
-        <v>442</v>
       </c>
       <c r="AB252" s="2">
         <v>44966</v>
@@ -14575,16 +14588,16 @@
         <v>12</v>
       </c>
       <c r="P253" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="R253" t="s">
         <v>7</v>
       </c>
       <c r="Z253" t="s">
+        <v>443</v>
+      </c>
+      <c r="AA253" t="s">
         <v>444</v>
-      </c>
-      <c r="AA253" t="s">
-        <v>445</v>
       </c>
       <c r="AB253" s="2">
         <v>44966</v>
@@ -14622,13 +14635,13 @@
         <v>12</v>
       </c>
       <c r="P254" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="R254" t="s">
         <v>7</v>
       </c>
       <c r="AA254" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="AB254" s="2">
         <v>44967</v>
@@ -14663,16 +14676,16 @@
         <v>12</v>
       </c>
       <c r="P255" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="R255" t="s">
         <v>7</v>
       </c>
       <c r="Z255" t="s">
+        <v>448</v>
+      </c>
+      <c r="AA255" t="s">
         <v>449</v>
-      </c>
-      <c r="AA255" t="s">
-        <v>450</v>
       </c>
       <c r="AB255" s="2">
         <v>44964</v>
@@ -14716,10 +14729,10 @@
         <v>7</v>
       </c>
       <c r="Z256" t="s">
+        <v>455</v>
+      </c>
+      <c r="AA256" t="s">
         <v>456</v>
-      </c>
-      <c r="AA256" t="s">
-        <v>457</v>
       </c>
       <c r="AB256" s="2">
         <v>44988</v>
@@ -14766,16 +14779,16 @@
         <v>12</v>
       </c>
       <c r="P257" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="R257" t="s">
         <v>7</v>
       </c>
       <c r="Z257" t="s">
+        <v>469</v>
+      </c>
+      <c r="AA257" t="s">
         <v>470</v>
-      </c>
-      <c r="AA257" t="s">
-        <v>471</v>
       </c>
       <c r="AB257" s="2">
         <v>45014</v>
@@ -14822,16 +14835,16 @@
         <v>12</v>
       </c>
       <c r="P258" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="R258" t="s">
         <v>7</v>
       </c>
       <c r="Z258" t="s">
+        <v>473</v>
+      </c>
+      <c r="AA258" t="s">
         <v>474</v>
-      </c>
-      <c r="AA258" t="s">
-        <v>475</v>
       </c>
       <c r="AB258" s="2">
         <v>45015</v>
@@ -14878,16 +14891,16 @@
         <v>12</v>
       </c>
       <c r="P259" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="R259" t="s">
         <v>7</v>
       </c>
       <c r="Z259" t="s">
+        <v>493</v>
+      </c>
+      <c r="AA259" t="s">
         <v>494</v>
-      </c>
-      <c r="AA259" t="s">
-        <v>495</v>
       </c>
       <c r="AB259" s="2">
         <v>45047</v>
@@ -14931,16 +14944,16 @@
         <v>12</v>
       </c>
       <c r="P260" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="R260" t="s">
         <v>7</v>
       </c>
       <c r="Z260" t="s">
+        <v>496</v>
+      </c>
+      <c r="AA260" t="s">
         <v>497</v>
-      </c>
-      <c r="AA260" t="s">
-        <v>498</v>
       </c>
       <c r="AB260" s="2">
         <v>45047</v>
@@ -14993,10 +15006,10 @@
         <v>7</v>
       </c>
       <c r="Z261" t="s">
+        <v>504</v>
+      </c>
+      <c r="AA261" t="s">
         <v>505</v>
-      </c>
-      <c r="AA261" t="s">
-        <v>506</v>
       </c>
       <c r="AB261" s="2">
         <v>44994</v>
@@ -15049,13 +15062,13 @@
         <v>7</v>
       </c>
       <c r="Z262" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="AB262" s="2">
         <v>44994</v>
       </c>
       <c r="AJ262" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
     </row>
     <row r="263" spans="1:36" x14ac:dyDescent="0.2">
@@ -15105,13 +15118,13 @@
         <v>7</v>
       </c>
       <c r="Z263" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="AB263" s="2">
         <v>44994</v>
       </c>
       <c r="AJ263" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="264" spans="1:36" x14ac:dyDescent="0.2">
@@ -15158,13 +15171,13 @@
         <v>7</v>
       </c>
       <c r="Z264" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="AB264" s="2">
         <v>44995</v>
       </c>
       <c r="AJ264" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="265" spans="1:36" x14ac:dyDescent="0.2">
@@ -15208,16 +15221,16 @@
         <v>12</v>
       </c>
       <c r="P265" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="R265" t="s">
         <v>7</v>
       </c>
       <c r="Z265" t="s">
+        <v>521</v>
+      </c>
+      <c r="AA265" t="s">
         <v>522</v>
-      </c>
-      <c r="AA265" t="s">
-        <v>523</v>
       </c>
       <c r="AB265" s="2">
         <v>45068</v>
@@ -15264,16 +15277,16 @@
         <v>12</v>
       </c>
       <c r="P266" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="R266" t="s">
         <v>7</v>
       </c>
       <c r="Z266" t="s">
+        <v>524</v>
+      </c>
+      <c r="AA266" t="s">
         <v>525</v>
-      </c>
-      <c r="AA266" t="s">
-        <v>526</v>
       </c>
       <c r="AB266" s="2">
         <v>45068</v>
@@ -15311,16 +15324,16 @@
         <v>12</v>
       </c>
       <c r="P267" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="R267" t="s">
         <v>7</v>
       </c>
       <c r="Z267" t="s">
+        <v>527</v>
+      </c>
+      <c r="AA267" t="s">
         <v>528</v>
-      </c>
-      <c r="AA267" t="s">
-        <v>529</v>
       </c>
       <c r="AB267" s="2">
         <v>45068</v>
@@ -15358,13 +15371,13 @@
         <v>12</v>
       </c>
       <c r="P268" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="R268" t="s">
         <v>7</v>
       </c>
       <c r="Z268" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="AB268" s="2">
         <v>45069</v>
@@ -15402,16 +15415,16 @@
         <v>12</v>
       </c>
       <c r="P269" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="R269" t="s">
         <v>7</v>
       </c>
       <c r="Z269" t="s">
+        <v>540</v>
+      </c>
+      <c r="AA269" t="s">
         <v>541</v>
-      </c>
-      <c r="AA269" t="s">
-        <v>542</v>
       </c>
       <c r="AB269" s="2">
         <v>45153</v>
@@ -15458,16 +15471,16 @@
         <v>12</v>
       </c>
       <c r="P270" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="R270" t="s">
         <v>7</v>
       </c>
       <c r="Z270" t="s">
+        <v>554</v>
+      </c>
+      <c r="AA270" t="s">
         <v>555</v>
-      </c>
-      <c r="AA270" t="s">
-        <v>556</v>
       </c>
       <c r="AB270" s="2">
         <v>45176</v>
@@ -15514,16 +15527,16 @@
         <v>12</v>
       </c>
       <c r="P271" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="R271" t="s">
         <v>7</v>
       </c>
       <c r="Z271" t="s">
+        <v>557</v>
+      </c>
+      <c r="AA271" t="s">
         <v>558</v>
-      </c>
-      <c r="AA271" t="s">
-        <v>559</v>
       </c>
       <c r="AB271" s="2">
         <v>45177</v>
@@ -15570,16 +15583,16 @@
         <v>12</v>
       </c>
       <c r="P272" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="R272" t="s">
         <v>7</v>
       </c>
       <c r="Z272" t="s">
+        <v>560</v>
+      </c>
+      <c r="AA272" t="s">
         <v>561</v>
-      </c>
-      <c r="AA272" t="s">
-        <v>562</v>
       </c>
       <c r="AB272" s="2">
         <v>45203</v>
@@ -15632,7 +15645,7 @@
         <v>7</v>
       </c>
       <c r="Z273" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="AB273" s="2">
         <v>45191</v>
@@ -15685,16 +15698,16 @@
         <v>7</v>
       </c>
       <c r="Z274" t="s">
+        <v>571</v>
+      </c>
+      <c r="AA274" t="s">
         <v>572</v>
-      </c>
-      <c r="AA274" t="s">
-        <v>573</v>
       </c>
       <c r="AB274" s="2">
         <v>45189</v>
       </c>
       <c r="AJ274" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
     </row>
     <row r="275" spans="1:36" x14ac:dyDescent="0.2">
@@ -15744,13 +15757,13 @@
         <v>7</v>
       </c>
       <c r="Z275" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="AB275" s="2">
         <v>45219</v>
       </c>
       <c r="AJ275" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="276" spans="1:36" x14ac:dyDescent="0.2">
@@ -15797,10 +15810,10 @@
         <v>7</v>
       </c>
       <c r="Z276" t="s">
+        <v>608</v>
+      </c>
+      <c r="AA276" t="s">
         <v>609</v>
-      </c>
-      <c r="AA276" t="s">
-        <v>610</v>
       </c>
       <c r="AB276" s="2">
         <v>45058</v>
@@ -15835,16 +15848,16 @@
         <v>12</v>
       </c>
       <c r="P277" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="R277" t="s">
         <v>7</v>
       </c>
       <c r="Z277" t="s">
+        <v>613</v>
+      </c>
+      <c r="AA277" t="s">
         <v>614</v>
-      </c>
-      <c r="AA277" t="s">
-        <v>615</v>
       </c>
       <c r="AB277" s="2">
         <v>45231</v>
@@ -15879,16 +15892,16 @@
         <v>12</v>
       </c>
       <c r="P278" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="R278" t="s">
         <v>7</v>
       </c>
       <c r="Z278" t="s">
+        <v>638</v>
+      </c>
+      <c r="AA278" t="s">
         <v>639</v>
-      </c>
-      <c r="AA278" t="s">
-        <v>640</v>
       </c>
       <c r="AB278" s="2">
         <v>45217</v>
@@ -15923,16 +15936,16 @@
         <v>12</v>
       </c>
       <c r="P279" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="R279" t="s">
         <v>7</v>
       </c>
       <c r="Z279" t="s">
+        <v>641</v>
+      </c>
+      <c r="AA279" t="s">
         <v>642</v>
-      </c>
-      <c r="AA279" t="s">
-        <v>643</v>
       </c>
       <c r="AB279" s="2">
         <v>45246</v>
@@ -15982,7 +15995,7 @@
         <v>7</v>
       </c>
       <c r="Z280" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
     </row>
     <row r="281" spans="1:36" x14ac:dyDescent="0.2">
@@ -16023,16 +16036,16 @@
         <v>12</v>
       </c>
       <c r="P281" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="R281" t="s">
         <v>7</v>
       </c>
       <c r="Z281" t="s">
+        <v>659</v>
+      </c>
+      <c r="AA281" t="s">
         <v>660</v>
-      </c>
-      <c r="AA281" t="s">
-        <v>661</v>
       </c>
       <c r="AB281" s="2">
         <v>45372</v>
@@ -16467,13 +16480,13 @@
         <v>12</v>
       </c>
       <c r="P290" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="R290" t="s">
         <v>14</v>
       </c>
       <c r="AJ290" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="291" spans="1:36" x14ac:dyDescent="0.2">
@@ -16517,13 +16530,13 @@
         <v>12</v>
       </c>
       <c r="P291" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="R291" t="s">
         <v>14</v>
       </c>
       <c r="AJ291" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="292" spans="1:36" x14ac:dyDescent="0.2">
@@ -16567,13 +16580,13 @@
         <v>12</v>
       </c>
       <c r="P292" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="R292" t="s">
         <v>14</v>
       </c>
       <c r="AJ292" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="293" spans="1:36" x14ac:dyDescent="0.2">
@@ -16620,7 +16633,7 @@
         <v>14</v>
       </c>
       <c r="AJ293" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="294" spans="1:36" x14ac:dyDescent="0.2">
@@ -16670,7 +16683,7 @@
         <v>14</v>
       </c>
       <c r="AJ294" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="295" spans="1:36" x14ac:dyDescent="0.2">
@@ -16714,13 +16727,13 @@
         <v>12</v>
       </c>
       <c r="P295" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="R295" t="s">
         <v>14</v>
       </c>
       <c r="AJ295" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="296" spans="1:36" x14ac:dyDescent="0.2">
@@ -16770,7 +16783,7 @@
         <v>14</v>
       </c>
       <c r="AJ296" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="297" spans="1:36" x14ac:dyDescent="0.2">
@@ -16814,7 +16827,7 @@
         <v>14</v>
       </c>
       <c r="AJ297" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="298" spans="1:36" x14ac:dyDescent="0.2">
@@ -16858,7 +16871,7 @@
         <v>14</v>
       </c>
       <c r="AJ298" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="299" spans="1:36" x14ac:dyDescent="0.2">
@@ -16902,13 +16915,13 @@
         <v>12</v>
       </c>
       <c r="P299" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="R299" t="s">
         <v>14</v>
       </c>
       <c r="AJ299" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="300" spans="1:36" x14ac:dyDescent="0.2">
@@ -16952,13 +16965,13 @@
         <v>12</v>
       </c>
       <c r="P300" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="R300" t="s">
         <v>14</v>
       </c>
       <c r="AJ300" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="301" spans="1:36" x14ac:dyDescent="0.2">
@@ -17008,7 +17021,7 @@
         <v>14</v>
       </c>
       <c r="AJ301" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="302" spans="1:36" x14ac:dyDescent="0.2">
@@ -17049,13 +17062,13 @@
         <v>12</v>
       </c>
       <c r="P302" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="R302" t="s">
         <v>14</v>
       </c>
       <c r="AJ302" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="303" spans="1:36" x14ac:dyDescent="0.2">
@@ -17105,7 +17118,7 @@
         <v>14</v>
       </c>
       <c r="AJ303" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="304" spans="1:36" x14ac:dyDescent="0.2">
@@ -17149,13 +17162,13 @@
         <v>12</v>
       </c>
       <c r="P304" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="R304" t="s">
         <v>14</v>
       </c>
       <c r="AJ304" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="305" spans="1:36" x14ac:dyDescent="0.2">
@@ -17205,7 +17218,7 @@
         <v>14</v>
       </c>
       <c r="AJ305" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="306" spans="1:36" x14ac:dyDescent="0.2">
@@ -17249,13 +17262,13 @@
         <v>12</v>
       </c>
       <c r="P306" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="R306" t="s">
         <v>14</v>
       </c>
       <c r="AJ306" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="307" spans="1:36" x14ac:dyDescent="0.2">
@@ -17269,10 +17282,10 @@
         <v>44906.786770833336</v>
       </c>
       <c r="D307" t="s">
+        <v>389</v>
+      </c>
+      <c r="E307" t="s">
         <v>390</v>
-      </c>
-      <c r="E307" t="s">
-        <v>391</v>
       </c>
       <c r="F307" t="s">
         <v>2</v>
@@ -17299,13 +17312,13 @@
         <v>12</v>
       </c>
       <c r="P307" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="R307" t="s">
         <v>14</v>
       </c>
       <c r="AJ307" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="308" spans="1:36" x14ac:dyDescent="0.2">
@@ -17355,7 +17368,7 @@
         <v>14</v>
       </c>
       <c r="AJ308" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="309" spans="1:36" x14ac:dyDescent="0.2">
@@ -17399,13 +17412,13 @@
         <v>12</v>
       </c>
       <c r="P309" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="R309" t="s">
         <v>14</v>
       </c>
       <c r="AJ309" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="310" spans="1:36" x14ac:dyDescent="0.2">
@@ -17449,13 +17462,13 @@
         <v>12</v>
       </c>
       <c r="P310" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="R310" t="s">
         <v>14</v>
       </c>
       <c r="AJ310" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="311" spans="1:36" x14ac:dyDescent="0.2">
@@ -17505,7 +17518,7 @@
         <v>14</v>
       </c>
       <c r="AJ311" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="312" spans="1:36" x14ac:dyDescent="0.2">
@@ -17555,7 +17568,7 @@
         <v>14</v>
       </c>
       <c r="AJ312" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="313" spans="1:36" x14ac:dyDescent="0.2">
@@ -17599,13 +17612,13 @@
         <v>12</v>
       </c>
       <c r="P313" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="R313" t="s">
         <v>14</v>
       </c>
       <c r="AJ313" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="314" spans="1:36" x14ac:dyDescent="0.2">
@@ -17649,7 +17662,7 @@
         <v>12</v>
       </c>
       <c r="P314" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="R314" t="s">
         <v>14</v>
@@ -17696,13 +17709,13 @@
         <v>12</v>
       </c>
       <c r="P315" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="R315" t="s">
         <v>14</v>
       </c>
       <c r="AJ315" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="316" spans="1:36" x14ac:dyDescent="0.2">
@@ -17752,7 +17765,7 @@
         <v>14</v>
       </c>
       <c r="AJ316" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
     </row>
     <row r="317" spans="1:36" x14ac:dyDescent="0.2">
@@ -17796,13 +17809,13 @@
         <v>12</v>
       </c>
       <c r="P317" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="R317" t="s">
         <v>14</v>
       </c>
       <c r="AJ317" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
     <row r="318" spans="1:36" x14ac:dyDescent="0.2">
@@ -17846,13 +17859,13 @@
         <v>12</v>
       </c>
       <c r="P318" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="R318" t="s">
         <v>14</v>
       </c>
       <c r="AJ318" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
     </row>
     <row r="319" spans="1:36" x14ac:dyDescent="0.2">
@@ -17896,13 +17909,13 @@
         <v>12</v>
       </c>
       <c r="P319" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="R319" t="s">
         <v>14</v>
       </c>
       <c r="AJ319" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
     </row>
     <row r="320" spans="1:36" x14ac:dyDescent="0.2">
@@ -17949,7 +17962,7 @@
         <v>14</v>
       </c>
       <c r="AJ320" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="321" spans="1:36" x14ac:dyDescent="0.2">
@@ -17993,13 +18006,13 @@
         <v>12</v>
       </c>
       <c r="P321" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="R321" t="s">
         <v>14</v>
       </c>
       <c r="AJ321" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
     </row>
     <row r="322" spans="1:36" x14ac:dyDescent="0.2">
@@ -18049,7 +18062,7 @@
         <v>14</v>
       </c>
       <c r="AJ322" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
     </row>
     <row r="323" spans="1:36" x14ac:dyDescent="0.2">
@@ -18099,7 +18112,7 @@
         <v>14</v>
       </c>
       <c r="AJ323" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="324" spans="1:36" x14ac:dyDescent="0.2">
@@ -18149,7 +18162,7 @@
         <v>14</v>
       </c>
       <c r="AJ324" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
     </row>
     <row r="325" spans="1:36" x14ac:dyDescent="0.2">
@@ -18199,7 +18212,7 @@
         <v>14</v>
       </c>
       <c r="AJ325" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
     <row r="326" spans="1:36" x14ac:dyDescent="0.2">
@@ -18293,7 +18306,7 @@
         <v>14</v>
       </c>
       <c r="AJ327" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
     </row>
     <row r="328" spans="1:36" x14ac:dyDescent="0.2">
@@ -18343,7 +18356,7 @@
         <v>14</v>
       </c>
       <c r="AJ328" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
     </row>
     <row r="329" spans="1:36" x14ac:dyDescent="0.2">
@@ -18387,13 +18400,13 @@
         <v>12</v>
       </c>
       <c r="P329" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="R329" t="s">
         <v>14</v>
       </c>
       <c r="AJ329" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="330" spans="1:36" x14ac:dyDescent="0.2">
@@ -18437,13 +18450,13 @@
         <v>12</v>
       </c>
       <c r="P330" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="R330" t="s">
         <v>14</v>
       </c>
       <c r="AJ330" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
     </row>
     <row r="331" spans="1:36" x14ac:dyDescent="0.2">
@@ -18487,13 +18500,13 @@
         <v>12</v>
       </c>
       <c r="P331" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="R331" t="s">
         <v>14</v>
       </c>
       <c r="AJ331" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
     </row>
     <row r="332" spans="1:36" x14ac:dyDescent="0.2">
@@ -18543,7 +18556,7 @@
         <v>14</v>
       </c>
       <c r="AJ332" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
     </row>
     <row r="333" spans="1:36" x14ac:dyDescent="0.2">
@@ -19234,8 +19247,8 @@
       <c r="W348" t="s">
         <v>180</v>
       </c>
-      <c r="X348" t="s">
-        <v>181</v>
+      <c r="X348" s="5" t="s">
+        <v>698</v>
       </c>
       <c r="Y348" s="2">
         <v>44715</v>
@@ -19273,10 +19286,10 @@
         <v>24</v>
       </c>
       <c r="W349" t="s">
+        <v>227</v>
+      </c>
+      <c r="X349" t="s">
         <v>228</v>
-      </c>
-      <c r="X349" t="s">
-        <v>229</v>
       </c>
       <c r="Y349" s="2">
         <v>44761</v>
@@ -19314,16 +19327,16 @@
         <v>12</v>
       </c>
       <c r="P350" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="R350" t="s">
         <v>24</v>
       </c>
       <c r="W350" t="s">
+        <v>244</v>
+      </c>
+      <c r="X350" t="s">
         <v>245</v>
-      </c>
-      <c r="X350" t="s">
-        <v>246</v>
       </c>
       <c r="Y350" s="2">
         <v>44825</v>
@@ -19364,16 +19377,16 @@
         <v>24</v>
       </c>
       <c r="W351" t="s">
+        <v>267</v>
+      </c>
+      <c r="X351" t="s">
         <v>268</v>
-      </c>
-      <c r="X351" t="s">
-        <v>269</v>
       </c>
       <c r="Y351" s="2">
         <v>44756</v>
       </c>
       <c r="AJ351" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="352" spans="1:36" x14ac:dyDescent="0.2">
@@ -19408,10 +19421,10 @@
         <v>24</v>
       </c>
       <c r="W352" t="s">
+        <v>279</v>
+      </c>
+      <c r="X352" t="s">
         <v>280</v>
-      </c>
-      <c r="X352" t="s">
-        <v>281</v>
       </c>
       <c r="Y352" s="2">
         <v>44741</v>
@@ -19449,10 +19462,10 @@
         <v>24</v>
       </c>
       <c r="W353" t="s">
+        <v>281</v>
+      </c>
+      <c r="X353" t="s">
         <v>282</v>
-      </c>
-      <c r="X353" t="s">
-        <v>283</v>
       </c>
       <c r="Y353" s="2">
         <v>44844</v>
@@ -19493,16 +19506,16 @@
         <v>24</v>
       </c>
       <c r="W354" t="s">
+        <v>308</v>
+      </c>
+      <c r="X354" t="s">
         <v>309</v>
-      </c>
-      <c r="X354" t="s">
-        <v>310</v>
       </c>
       <c r="Y354" s="2">
         <v>44851</v>
       </c>
       <c r="AJ354" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="355" spans="1:36" x14ac:dyDescent="0.2">
@@ -19537,22 +19550,22 @@
         <v>12</v>
       </c>
       <c r="P355" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R355" t="s">
         <v>24</v>
       </c>
       <c r="W355" t="s">
+        <v>326</v>
+      </c>
+      <c r="X355" t="s">
         <v>327</v>
-      </c>
-      <c r="X355" t="s">
-        <v>328</v>
       </c>
       <c r="Y355" s="2">
         <v>44866</v>
       </c>
       <c r="AJ355" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="356" spans="1:36" x14ac:dyDescent="0.2">
@@ -19590,16 +19603,16 @@
         <v>24</v>
       </c>
       <c r="W356" t="s">
+        <v>337</v>
+      </c>
+      <c r="X356" t="s">
         <v>338</v>
-      </c>
-      <c r="X356" t="s">
-        <v>339</v>
       </c>
       <c r="Y356" s="2">
         <v>44866</v>
       </c>
       <c r="AJ356" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="357" spans="1:36" x14ac:dyDescent="0.2">
@@ -19634,10 +19647,10 @@
         <v>24</v>
       </c>
       <c r="W357" t="s">
+        <v>357</v>
+      </c>
+      <c r="X357" t="s">
         <v>358</v>
-      </c>
-      <c r="X357" t="s">
-        <v>359</v>
       </c>
       <c r="Y357" s="2">
         <v>44713</v>
@@ -19675,16 +19688,16 @@
         <v>24</v>
       </c>
       <c r="W358" t="s">
+        <v>363</v>
+      </c>
+      <c r="X358" t="s">
         <v>364</v>
-      </c>
-      <c r="X358" t="s">
-        <v>365</v>
       </c>
       <c r="Y358" s="2">
         <v>44748</v>
       </c>
       <c r="AJ358" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="359" spans="1:36" x14ac:dyDescent="0.2">
@@ -19719,16 +19732,16 @@
         <v>24</v>
       </c>
       <c r="W359" t="s">
+        <v>366</v>
+      </c>
+      <c r="X359" t="s">
         <v>367</v>
-      </c>
-      <c r="X359" t="s">
-        <v>368</v>
       </c>
       <c r="Y359" s="2">
         <v>44690</v>
       </c>
       <c r="AJ359" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="360" spans="1:36" x14ac:dyDescent="0.2">
@@ -19763,16 +19776,16 @@
         <v>24</v>
       </c>
       <c r="W360" t="s">
+        <v>372</v>
+      </c>
+      <c r="X360" t="s">
         <v>373</v>
-      </c>
-      <c r="X360" t="s">
-        <v>374</v>
       </c>
       <c r="Y360" s="2">
         <v>44594</v>
       </c>
       <c r="AJ360" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="361" spans="1:36" x14ac:dyDescent="0.2">
@@ -19804,22 +19817,22 @@
         <v>12</v>
       </c>
       <c r="P361" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="R361" t="s">
         <v>24</v>
       </c>
       <c r="W361" t="s">
+        <v>376</v>
+      </c>
+      <c r="X361" t="s">
         <v>377</v>
-      </c>
-      <c r="X361" t="s">
-        <v>378</v>
       </c>
       <c r="Y361" s="2">
         <v>44287</v>
       </c>
       <c r="AJ361" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="362" spans="1:36" x14ac:dyDescent="0.2">
@@ -19854,16 +19867,16 @@
         <v>24</v>
       </c>
       <c r="W362" t="s">
+        <v>379</v>
+      </c>
+      <c r="X362" t="s">
         <v>380</v>
-      </c>
-      <c r="X362" t="s">
-        <v>381</v>
       </c>
       <c r="Y362" s="2">
         <v>44154</v>
       </c>
       <c r="AJ362" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="363" spans="1:36" x14ac:dyDescent="0.2">
@@ -19895,22 +19908,22 @@
         <v>12</v>
       </c>
       <c r="P363" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="R363" t="s">
         <v>24</v>
       </c>
       <c r="W363" t="s">
+        <v>382</v>
+      </c>
+      <c r="X363" t="s">
         <v>383</v>
-      </c>
-      <c r="X363" t="s">
-        <v>384</v>
       </c>
       <c r="Y363" s="2">
         <v>44719</v>
       </c>
       <c r="AJ363" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="364" spans="1:36" x14ac:dyDescent="0.2">
@@ -19945,10 +19958,10 @@
         <v>24</v>
       </c>
       <c r="W364" t="s">
+        <v>488</v>
+      </c>
+      <c r="X364" t="s">
         <v>489</v>
-      </c>
-      <c r="X364" t="s">
-        <v>490</v>
       </c>
       <c r="Y364" s="2">
         <v>45009</v>
@@ -19986,10 +19999,10 @@
         <v>24</v>
       </c>
       <c r="W365" t="s">
+        <v>490</v>
+      </c>
+      <c r="X365" t="s">
         <v>491</v>
-      </c>
-      <c r="X365" t="s">
-        <v>492</v>
       </c>
       <c r="Y365" s="2">
         <v>44845</v>
@@ -20030,10 +20043,10 @@
         <v>24</v>
       </c>
       <c r="W366" t="s">
+        <v>518</v>
+      </c>
+      <c r="X366" t="s">
         <v>519</v>
-      </c>
-      <c r="X366" t="s">
-        <v>520</v>
       </c>
       <c r="Y366" s="2">
         <v>45065</v>
@@ -20071,16 +20084,16 @@
         <v>12</v>
       </c>
       <c r="P367" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="R367" t="s">
         <v>24</v>
       </c>
       <c r="W367" t="s">
+        <v>535</v>
+      </c>
+      <c r="X367" t="s">
         <v>536</v>
-      </c>
-      <c r="X367" t="s">
-        <v>537</v>
       </c>
       <c r="Y367" s="2">
         <v>45092</v>
@@ -20118,16 +20131,16 @@
         <v>24</v>
       </c>
       <c r="W368" t="s">
+        <v>562</v>
+      </c>
+      <c r="X368" t="s">
         <v>563</v>
-      </c>
-      <c r="X368" t="s">
-        <v>564</v>
       </c>
       <c r="Y368" s="2">
         <v>45047</v>
       </c>
       <c r="AJ368" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="369" spans="1:36" x14ac:dyDescent="0.2">
@@ -20162,10 +20175,10 @@
         <v>24</v>
       </c>
       <c r="W369" t="s">
+        <v>565</v>
+      </c>
+      <c r="X369" t="s">
         <v>566</v>
-      </c>
-      <c r="X369" t="s">
-        <v>567</v>
       </c>
       <c r="Y369" s="2">
         <v>45195</v>
@@ -20203,10 +20216,10 @@
         <v>24</v>
       </c>
       <c r="W370" t="s">
+        <v>578</v>
+      </c>
+      <c r="X370" t="s">
         <v>579</v>
-      </c>
-      <c r="X370" t="s">
-        <v>580</v>
       </c>
       <c r="Y370" s="2">
         <v>45159</v>
@@ -20244,10 +20257,10 @@
         <v>24</v>
       </c>
       <c r="W371" t="s">
+        <v>581</v>
+      </c>
+      <c r="X371" t="s">
         <v>582</v>
-      </c>
-      <c r="X371" t="s">
-        <v>583</v>
       </c>
       <c r="Y371" s="2">
         <v>45196</v>
@@ -20285,10 +20298,10 @@
         <v>24</v>
       </c>
       <c r="W372" t="s">
+        <v>583</v>
+      </c>
+      <c r="X372" t="s">
         <v>584</v>
-      </c>
-      <c r="X372" t="s">
-        <v>585</v>
       </c>
       <c r="Y372" s="2">
         <v>45078</v>
@@ -20326,10 +20339,10 @@
         <v>24</v>
       </c>
       <c r="W373" t="s">
+        <v>585</v>
+      </c>
+      <c r="X373" t="s">
         <v>586</v>
-      </c>
-      <c r="X373" t="s">
-        <v>587</v>
       </c>
       <c r="Y373" s="2">
         <v>45170</v>
@@ -20367,10 +20380,10 @@
         <v>24</v>
       </c>
       <c r="W374" t="s">
+        <v>587</v>
+      </c>
+      <c r="X374" t="s">
         <v>588</v>
-      </c>
-      <c r="X374" t="s">
-        <v>589</v>
       </c>
       <c r="Y374" s="2">
         <v>44440</v>
@@ -20408,16 +20421,16 @@
         <v>24</v>
       </c>
       <c r="W375" t="s">
+        <v>591</v>
+      </c>
+      <c r="X375" t="s">
         <v>592</v>
-      </c>
-      <c r="X375" t="s">
-        <v>593</v>
       </c>
       <c r="Y375" s="2">
         <v>45112</v>
       </c>
       <c r="AJ375" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
     </row>
     <row r="376" spans="1:36" x14ac:dyDescent="0.2">
@@ -20452,10 +20465,10 @@
         <v>24</v>
       </c>
       <c r="W376" t="s">
+        <v>597</v>
+      </c>
+      <c r="X376" t="s">
         <v>598</v>
-      </c>
-      <c r="X376" t="s">
-        <v>599</v>
       </c>
       <c r="Y376" s="2">
         <v>45211</v>
@@ -20493,16 +20506,16 @@
         <v>12</v>
       </c>
       <c r="P377" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="R377" t="s">
         <v>24</v>
       </c>
       <c r="W377" t="s">
+        <v>616</v>
+      </c>
+      <c r="X377" t="s">
         <v>617</v>
-      </c>
-      <c r="X377" t="s">
-        <v>618</v>
       </c>
       <c r="Y377" s="2">
         <v>45237</v>
@@ -20543,16 +20556,16 @@
         <v>24</v>
       </c>
       <c r="W378" t="s">
+        <v>634</v>
+      </c>
+      <c r="X378" t="s">
         <v>635</v>
-      </c>
-      <c r="X378" t="s">
-        <v>636</v>
       </c>
       <c r="Y378" s="2">
         <v>45260</v>
       </c>
       <c r="AJ378" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
     </row>
     <row r="379" spans="1:36" x14ac:dyDescent="0.2">
@@ -20599,19 +20612,19 @@
         <v>49</v>
       </c>
       <c r="R379" t="s">
+        <v>214</v>
+      </c>
+      <c r="S379" t="s">
         <v>215</v>
       </c>
-      <c r="S379" t="s">
+      <c r="T379">
+        <v>3</v>
+      </c>
+      <c r="U379" t="s">
         <v>216</v>
       </c>
-      <c r="T379">
-        <v>3</v>
-      </c>
-      <c r="U379" t="s">
+      <c r="AG379" t="s">
         <v>217</v>
-      </c>
-      <c r="AG379" t="s">
-        <v>218</v>
       </c>
       <c r="AH379">
         <v>1</v>
@@ -20620,7 +20633,7 @@
         <v>43</v>
       </c>
       <c r="AJ379" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="380" spans="1:36" x14ac:dyDescent="0.2">
@@ -20667,22 +20680,22 @@
         <v>49</v>
       </c>
       <c r="R380" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="S380" t="s">
+        <v>302</v>
+      </c>
+      <c r="T380">
+        <v>3</v>
+      </c>
+      <c r="U380" t="s">
         <v>303</v>
       </c>
-      <c r="T380">
-        <v>3</v>
-      </c>
-      <c r="U380" t="s">
+      <c r="V380">
+        <v>3</v>
+      </c>
+      <c r="AJ380" t="s">
         <v>304</v>
-      </c>
-      <c r="V380">
-        <v>3</v>
-      </c>
-      <c r="AJ380" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="381" spans="1:36" x14ac:dyDescent="0.2">
@@ -20729,22 +20742,22 @@
         <v>49</v>
       </c>
       <c r="R381" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="S381" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="T381">
         <v>4</v>
       </c>
       <c r="U381" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="V381">
         <v>2</v>
       </c>
       <c r="AJ381" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="382" spans="1:36" x14ac:dyDescent="0.2">
@@ -20791,22 +20804,22 @@
         <v>34</v>
       </c>
       <c r="R382" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="S382" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="T382">
         <v>10</v>
       </c>
       <c r="U382" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="V382">
         <v>2</v>
       </c>
       <c r="AJ382" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="383" spans="1:36" x14ac:dyDescent="0.2">
@@ -20853,22 +20866,22 @@
         <v>49</v>
       </c>
       <c r="R383" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="S383" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="T383">
         <v>8</v>
       </c>
       <c r="U383" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="V383">
         <v>1</v>
       </c>
       <c r="AJ383" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="384" spans="1:36" x14ac:dyDescent="0.2">
@@ -20915,22 +20928,22 @@
         <v>49</v>
       </c>
       <c r="R384" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="S384" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="T384">
         <v>4</v>
       </c>
       <c r="U384" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="V384">
         <v>2</v>
       </c>
       <c r="AJ384" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="385" spans="1:36" x14ac:dyDescent="0.2">
@@ -20974,25 +20987,25 @@
         <v>12</v>
       </c>
       <c r="P385" t="s">
+        <v>386</v>
+      </c>
+      <c r="R385" t="s">
+        <v>214</v>
+      </c>
+      <c r="S385" t="s">
         <v>387</v>
       </c>
-      <c r="R385" t="s">
-        <v>215</v>
-      </c>
-      <c r="S385" t="s">
-        <v>388</v>
-      </c>
       <c r="T385">
         <v>2</v>
       </c>
       <c r="U385" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="V385">
         <v>1</v>
       </c>
       <c r="AJ385" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="386" spans="1:36" x14ac:dyDescent="0.2">
@@ -21006,10 +21019,10 @@
         <v>44906.819293981483</v>
       </c>
       <c r="D386" t="s">
+        <v>389</v>
+      </c>
+      <c r="E386" t="s">
         <v>390</v>
-      </c>
-      <c r="E386" t="s">
-        <v>391</v>
       </c>
       <c r="F386" t="s">
         <v>2</v>
@@ -21036,28 +21049,28 @@
         <v>49</v>
       </c>
       <c r="R386" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="S386" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="T386">
         <v>10</v>
       </c>
       <c r="U386" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="AG386" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="AH386">
         <v>1</v>
       </c>
       <c r="AI386" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="AJ386" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="387" spans="1:36" x14ac:dyDescent="0.2">
@@ -21071,10 +21084,10 @@
         <v>44906.824050925927</v>
       </c>
       <c r="D387" t="s">
+        <v>389</v>
+      </c>
+      <c r="E387" t="s">
         <v>390</v>
-      </c>
-      <c r="E387" t="s">
-        <v>391</v>
       </c>
       <c r="F387" t="s">
         <v>2</v>
@@ -21101,13 +21114,13 @@
         <v>49</v>
       </c>
       <c r="R387" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="U387" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="AJ387" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="388" spans="1:36" x14ac:dyDescent="0.2">
@@ -21121,10 +21134,10 @@
         <v>44906.84783564815</v>
       </c>
       <c r="D388" t="s">
+        <v>389</v>
+      </c>
+      <c r="E388" t="s">
         <v>390</v>
-      </c>
-      <c r="E388" t="s">
-        <v>391</v>
       </c>
       <c r="F388" t="s">
         <v>2</v>
@@ -21151,10 +21164,10 @@
         <v>49</v>
       </c>
       <c r="R388" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="AJ388" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="389" spans="1:36" x14ac:dyDescent="0.2">
@@ -21198,22 +21211,22 @@
         <v>23</v>
       </c>
       <c r="R389" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="S389" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="T389">
         <v>1</v>
       </c>
       <c r="U389" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="V389">
         <v>2</v>
       </c>
       <c r="AJ389" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="390" spans="1:36" x14ac:dyDescent="0.2">
@@ -21260,28 +21273,28 @@
         <v>49</v>
       </c>
       <c r="R390" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="S390" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="T390">
         <v>4</v>
       </c>
       <c r="U390" t="s">
+        <v>216</v>
+      </c>
+      <c r="AG390" t="s">
         <v>217</v>
-      </c>
-      <c r="AG390" t="s">
-        <v>218</v>
       </c>
       <c r="AH390">
         <v>1</v>
       </c>
       <c r="AI390" t="s">
+        <v>484</v>
+      </c>
+      <c r="AJ390" t="s">
         <v>485</v>
-      </c>
-      <c r="AJ390" t="s">
-        <v>486</v>
       </c>
     </row>
     <row r="391" spans="1:36" x14ac:dyDescent="0.2">
@@ -21325,22 +21338,22 @@
         <v>49</v>
       </c>
       <c r="R391" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="S391" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="T391">
         <v>150</v>
       </c>
       <c r="U391" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="V391">
         <v>1</v>
       </c>
       <c r="AJ391" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
     </row>
     <row r="392" spans="1:36" x14ac:dyDescent="0.2">
@@ -21384,25 +21397,25 @@
         <v>5</v>
       </c>
       <c r="Q392" t="s">
+        <v>652</v>
+      </c>
+      <c r="R392" t="s">
+        <v>214</v>
+      </c>
+      <c r="S392" t="s">
         <v>653</v>
       </c>
-      <c r="R392" t="s">
-        <v>215</v>
-      </c>
-      <c r="S392" t="s">
-        <v>654</v>
-      </c>
       <c r="T392">
         <v>3</v>
       </c>
       <c r="U392" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="V392">
         <v>1</v>
       </c>
       <c r="AJ392" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
     </row>
   </sheetData>
@@ -21411,6 +21424,9 @@
       <sortCondition descending="1" ref="AE1:AE392"/>
     </sortState>
   </autoFilter>
+  <hyperlinks>
+    <hyperlink ref="X348" r:id="rId1" xr:uid="{F86AD19A-5CDC-7E41-A02F-AD3EB0F722A9}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>